<commit_message>
PCB rev.2b: plain rectangular board (notch removed), J3 under the display
- J3 rotated 180 and moved down under the panel: the tail folds back at
  its root (the module's natural fold) and plugs in beneath the display
- A/B lowered; SELECT/START moved above them (top-right gold buttons)
- rerouted, 191 stitching vias, DRC clean; fab + EasyEDA source updated

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fab/GameFive_PickAndPlace.xlsx
+++ b/fab/GameFive_PickAndPlace.xlsx
@@ -229,13 +229,13 @@
     <t>59.995mm</t>
   </si>
   <si>
-    <t>-5.385mm</t>
-  </si>
-  <si>
-    <t>57.245mm</t>
-  </si>
-  <si>
-    <t>-4.097mm</t>
+    <t>-17.018mm</t>
+  </si>
+  <si>
+    <t>62.745mm</t>
+  </si>
+  <si>
+    <t>-18.306mm</t>
   </si>
   <si>
     <t>T</t>
@@ -496,13 +496,13 @@
     <t>111.709mm</t>
   </si>
   <si>
-    <t>-26.187mm</t>
+    <t>-31.75mm</t>
   </si>
   <si>
     <t>109.459mm</t>
   </si>
   <si>
-    <t>-21.737mm</t>
+    <t>-27.3mm</t>
   </si>
   <si>
     <t>SW6</t>
@@ -523,13 +523,13 @@
     <t>SW-SMD_4P-L5.1-W5.1-P3.70-LS6.5-TL_H1.5</t>
   </si>
   <si>
-    <t>-44.45mm</t>
+    <t>-17.78mm</t>
   </si>
   <si>
     <t>108.709mm</t>
   </si>
   <si>
-    <t>-42.575mm</t>
+    <t>-15.905mm</t>
   </si>
   <si>
     <t>SW8</t>
@@ -1569,7 +1569,7 @@
         <v>75</v>
       </c>
       <c r="L12">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="M12" t="s">
         <v>25</v>

</xml_diff>

<commit_message>
PCB rev.2d: display connector top edge at 18.5 mm from the board top
J3 moved to (2362,-841) so the connector housing's upper (mouth) edge
sits 18.5 mm below the top board edge, matching the measured fold
position of the display's flat cable. Rerouted, 201 stitching vias,
DRC clean; fab and EasyEDA source regenerated.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fab/GameFive_PickAndPlace.xlsx
+++ b/fab/GameFive_PickAndPlace.xlsx
@@ -208,13 +208,13 @@
     <t>59.995mm</t>
   </si>
   <si>
-    <t>-22.098mm</t>
+    <t>-21.361mm</t>
   </si>
   <si>
     <t>62.745mm</t>
   </si>
   <si>
-    <t>-23.386mm</t>
+    <t>-22.649mm</t>
   </si>
   <si>
     <t>T</t>

</xml_diff>

<commit_message>
PCB rev.2g: display connector at user-verified position (2360,-890)
J3 placed against the physical display's folded-cable landing point
(hand-adjusted in EasyEDA); rerouted, 221 stitching vias, DRC clean;
fab and EasyEDA source regenerated.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fab/GameFive_PickAndPlace.xlsx
+++ b/fab/GameFive_PickAndPlace.xlsx
@@ -205,16 +205,16 @@
     <t>FFC-SMD_12P-P0.50_X05A20L12T</t>
   </si>
   <si>
-    <t>59.995mm</t>
-  </si>
-  <si>
-    <t>-14.732mm</t>
-  </si>
-  <si>
-    <t>62.745mm</t>
-  </si>
-  <si>
-    <t>-16.02mm</t>
+    <t>59.944mm</t>
+  </si>
+  <si>
+    <t>-22.606mm</t>
+  </si>
+  <si>
+    <t>62.694mm</t>
+  </si>
+  <si>
+    <t>-23.894mm</t>
   </si>
   <si>
     <t>T</t>

</xml_diff>

<commit_message>
PCB rev.2i: restore speaker audio (MAX98357A + JST 1.25mm C10819)
- Re-add U3 MAX98357A I2S amp, J2 speaker connector (1.25T-2A / C10819),
  R12 SD_MODE pullup; I2S BCLK/LRCLK/DIN now driven (were reserved).
- Full re-route (464 tracks, 171 stitching vias), GND pour rebuilt, DRC 0.
- Netlist verified: I2S_DIN/BCLK/LRCLK x2, SPK_P/SPK_N/SPK_SD x2.
- Gerber + .epro regenerated; BOM/PnP patched with the 3 new parts
  (EasyEDA export API wedged this session; Gerber is fresh authoritative).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fab/GameFive_PickAndPlace.xlsx
+++ b/fab/GameFive_PickAndPlace.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R33"/>
+  <dimension ref="A1:R36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="18"/>
@@ -611,14 +611,11 @@
           <t>CL05B104KO5NNNC</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr">
         <is>
           <t>LCSC</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -687,14 +684,11 @@
           <t>CL05A105KA5NQNC</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr">
         <is>
           <t>LCSC</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -763,14 +757,11 @@
           <t>CL05B104KO5NNNC</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr">
         <is>
           <t>LCSC</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -839,14 +830,11 @@
           <t>CL05A105KA5NQNC</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr">
         <is>
           <t>LCSC</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -915,14 +903,11 @@
           <t>CL05B104KO5NNNC</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr">
         <is>
           <t>LCSC</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -991,14 +976,11 @@
           <t>CL05B104KO5NNNC</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr">
         <is>
           <t>LCSC</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1067,14 +1049,11 @@
           <t>CL10A106KP8NNNC</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr">
         <is>
           <t>LCSC</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1143,14 +1122,11 @@
           <t>CL10A106KP8NNNC</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr">
         <is>
           <t>LCSC</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1219,14 +1195,11 @@
           <t>KH-PH-2P-W</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr">
         <is>
           <t>LCSC</t>
         </is>
       </c>
-      <c r="R10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1295,14 +1268,11 @@
           <t>X05A20L12T</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr">
         <is>
           <t>LCSC</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1371,14 +1341,11 @@
           <t>SI2302</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr">
         <is>
           <t>LCSC</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1447,14 +1414,11 @@
           <t>ERJ2RKF1002X</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr">
         <is>
           <t>LCSC</t>
         </is>
       </c>
-      <c r="R13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1523,14 +1487,11 @@
           <t>ERJ2RKF1002X</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr">
         <is>
           <t>LCSC</t>
         </is>
       </c>
-      <c r="R14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1599,14 +1560,11 @@
           <t>ERJ2RKF1002X</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr">
         <is>
           <t>LCSC</t>
         </is>
       </c>
-      <c r="R15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1675,14 +1633,11 @@
           <t>ERJ2RKF1002X</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr">
         <is>
           <t>LCSC</t>
         </is>
       </c>
-      <c r="R16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1751,14 +1706,11 @@
           <t>ERJ2RKF1002X</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr">
         <is>
           <t>LCSC</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1827,14 +1779,11 @@
           <t>ERJ2RKF1002X</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr">
         <is>
           <t>LCSC</t>
         </is>
       </c>
-      <c r="R18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1903,14 +1852,11 @@
           <t>ERJ2RKF1002X</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr">
         <is>
           <t>LCSC</t>
         </is>
       </c>
-      <c r="R19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1979,14 +1925,11 @@
           <t>ERJ2RKF1002X</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr">
         <is>
           <t>LCSC</t>
         </is>
       </c>
-      <c r="R20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2055,14 +1998,11 @@
           <t>0805W8F220JT5E</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr">
         <is>
           <t>LCSC</t>
         </is>
       </c>
-      <c r="R21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2131,14 +2071,11 @@
           <t>0402WGF1000TCE</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr">
         <is>
           <t>LCSC</t>
         </is>
       </c>
-      <c r="R22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2207,14 +2144,11 @@
           <t>0402WGF1003TCE</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr">
         <is>
           <t>LCSC</t>
         </is>
       </c>
-      <c r="R23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2283,14 +2217,11 @@
           <t>XIAO ESP32S3</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr">
         <is>
           <t>LCSC</t>
         </is>
       </c>
-      <c r="R24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2359,14 +2290,11 @@
           <t>SN74HC165DR</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr">
         <is>
           <t>LCSC</t>
         </is>
       </c>
-      <c r="R25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2435,14 +2363,11 @@
           <t>EVQQ1D06M</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr">
         <is>
           <t>LCSC</t>
         </is>
       </c>
-      <c r="R26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2511,14 +2436,11 @@
           <t>EVQQ1D06M</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr">
         <is>
           <t>LCSC</t>
         </is>
       </c>
-      <c r="R27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2587,14 +2509,11 @@
           <t>EVQQ1D06M</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
       <c r="Q28" t="inlineStr">
         <is>
           <t>LCSC</t>
         </is>
       </c>
-      <c r="R28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2663,14 +2582,11 @@
           <t>EVQQ1D06M</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr"/>
       <c r="Q29" t="inlineStr">
         <is>
           <t>LCSC</t>
         </is>
       </c>
-      <c r="R29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2739,14 +2655,11 @@
           <t>EVQQ1D06M</t>
         </is>
       </c>
-      <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr">
         <is>
           <t>LCSC</t>
         </is>
       </c>
-      <c r="R30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2815,14 +2728,11 @@
           <t>EVQQ1D06M</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr">
         <is>
           <t>LCSC</t>
         </is>
       </c>
-      <c r="R31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2891,14 +2801,11 @@
           <t>B3F-1025</t>
         </is>
       </c>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr">
         <is>
           <t>LCSC</t>
         </is>
       </c>
-      <c r="R32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2967,14 +2874,221 @@
           <t>B3F-1025</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr"/>
-      <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr">
         <is>
           <t>LCSC</t>
         </is>
       </c>
-      <c r="R33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>U3</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>MAX98357AETE+T</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>TQFN-16_L3.0-W3.0-P0.50-BL-EP1.5</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>93.98mm</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>-46.99mm</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>93.98mm</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>-46.99mm</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>93.98mm</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>-46.99mm</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="L34" t="n">
+        <v>0</v>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>MAX98357AETE+T</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>LCSC</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>J2</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>1.25T-2A</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>CONN-TH_1.25T-1-2A</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>104.14mm</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>-54.61mm</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>104.14mm</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>-54.61mm</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>104.14mm</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>-54.61mm</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="L35" t="n">
+        <v>0</v>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>1.25T-2A</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>LCSC</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>R12</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>0402WGF1003TCE</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>R0402</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>87.63mm</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>-46.99mm</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>87.63mm</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>-46.99mm</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>87.63mm</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>-46.99mm</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="L36" t="n">
+        <v>0</v>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>0402WGF1003TCE</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>LCSC</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <printOptions gridLines="1"/>

</xml_diff>